<commit_message>
fix: use clearly fictional sample data and address bugbot findings
Replace all real-world registry names, organization names, project IDs,
and URLs with obviously fictional "Example"/"Sample" prefixed values so
the test fixtures cannot be mistaken for real data. Picklist enum values
(projectSector, projectType, projectStatus, ratingType, etc.) are kept
as valid governance entries.

Bugbot fixes:
- remove unused PLACEHOLDER_VERIFICATION_ID and
  PLACEHOLDER_PROJECT_METHODOLOGY_ID constants
- fix Unit 1 unitCount from 4000 to 4001 (inclusive range 1000-5000)
- fix Gold Standard label linkage from UNIT_1 to UNIT_3
</commit_message>
<xml_diff>
--- a/tests/v2/live-api/data/sample-projects-import.xlsx
+++ b/tests/v2/live-api/data/sample-projects-import.xlsx
@@ -450,22 +450,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>VCS</v>
+        <v>Sample Global Registry</v>
       </c>
       <c r="B2" t="str">
-        <v>VCS-2024-001</v>
+        <v>SAMPLE-PRJ-2024-001</v>
       </c>
       <c r="C2" t="str">
-        <v>Verified Carbon Standard</v>
+        <v>Example Crediting Program A</v>
       </c>
       <c r="D2" t="str">
-        <v>Mekong Delta Mangrove Restoration</v>
+        <v>Example Mangrove Restoration Project</v>
       </c>
       <c r="E2" t="str">
-        <v>https://registry.verra.org/app/projectDetail/VCS/2024001</v>
+        <v>https://example.com/registry/projects/sample-prj-2024-001</v>
       </c>
       <c r="F2" t="str">
-        <v>Large-scale mangrove restoration project across 5,000 hectares in the Mekong Delta region of Vietnam, combining reforestation with community-based sustainable aquaculture. The project protects biodiversity corridors and strengthens coastal resilience against typhoons and sea-level rise.</v>
+        <v>Sample large-scale mangrove restoration project for testing purposes. This fictional project demonstrates a reforestation scenario with community-based sustainable aquaculture across an example coastal region.</v>
       </c>
       <c r="G2" t="str">
         <v>["Afforestation and reforestation"]</v>
@@ -488,16 +488,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Gold Standard</v>
+        <v>Example Standards Body</v>
       </c>
       <c r="B3" t="str">
-        <v>GS-10542</v>
+        <v>SAMPLE-PRJ-2024-002</v>
       </c>
       <c r="D3" t="str">
-        <v>Gujarat Solar Cookstove Distribution</v>
+        <v>Sample Solar Cookstove Distribution</v>
       </c>
       <c r="E3" t="str">
-        <v>https://registry.goldstandard.org/projects/details/10542</v>
+        <v>https://example.com/registry/projects/sample-prj-2024-002</v>
       </c>
       <c r="G3" t="str">
         <v>["Energy demand"]</v>
@@ -517,22 +517,22 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>CAR</v>
+        <v>Example Forestry Registry</v>
       </c>
       <c r="B4" t="str">
-        <v>CAR-2025-078</v>
+        <v>SAMPLE-PRJ-2025-003</v>
       </c>
       <c r="C4" t="str">
-        <v>Climate Action Reserve</v>
+        <v>Example Crediting Program B</v>
       </c>
       <c r="D4" t="str">
-        <v>Pacific Northwest Improved Forest Management</v>
+        <v>Example Improved Forest Management</v>
       </c>
       <c r="E4" t="str">
-        <v>https://www.climateactionreserve.org/how/protocols/forest/2025-078</v>
+        <v>https://example.com/registry/projects/sample-prj-2025-003</v>
       </c>
       <c r="F4" t="str">
-        <v>Improved forest management across 12,000 acres of mixed-conifer forest in Oregon. The project transitions from conventional harvest rotations to extended rotations and selective thinning, increasing above-ground carbon stocks by 35% over the crediting period.</v>
+        <v>Sample improved forest management project for testing. This fictional project demonstrates extended rotations and selective thinning in a mixed-conifer forest scenario for CADT import/export testing.</v>
       </c>
       <c r="G4" t="str">
         <v>["Afforestation and reforestation","Agriculture"]</v>
@@ -592,7 +592,7 @@
         <v>Viet Nam</v>
       </c>
       <c r="B2" t="str">
-        <v>Mekong Delta</v>
+        <v>Example Delta Region</v>
       </c>
       <c r="C2" t="str">
         <v>{"type":"Point","coordinates":[105.7,9.8]}</v>
@@ -601,7 +601,7 @@
         <v>GeoJSON</v>
       </c>
       <c r="E2" t="str">
-        <v>https://example.com/maps/mekong-delta-mangrove.geojson</v>
+        <v>https://example.com/maps/sample-mangrove.geojson</v>
       </c>
       <c r="F2" t="str">
         <v>NEW-1</v>
@@ -612,7 +612,7 @@
         <v>Viet Nam</v>
       </c>
       <c r="B3" t="str">
-        <v>Ca Mau Province</v>
+        <v>Example Province</v>
       </c>
       <c r="C3" t="str">
         <v>{"type":"Point","coordinates":[104.98,8.98]}</v>
@@ -629,7 +629,7 @@
         <v>India</v>
       </c>
       <c r="B4" t="str">
-        <v>Gujarat</v>
+        <v>Example State</v>
       </c>
       <c r="C4" t="str">
         <v>POINT(72.57 23.03)</v>
@@ -638,7 +638,7 @@
         <v>GeoJSON</v>
       </c>
       <c r="E4" t="str">
-        <v>https://example.com/maps/gujarat-solar.geojson</v>
+        <v>https://example.com/maps/sample-solar.geojson</v>
       </c>
       <c r="F4" t="str">
         <v>NEW-2</v>
@@ -649,7 +649,7 @@
         <v>United States of America</v>
       </c>
       <c r="B5" t="str">
-        <v>Oregon</v>
+        <v>Example State</v>
       </c>
       <c r="C5" t="str">
         <v>{"type":"Polygon","coordinates":[[[-122.5,44.0],[-121.5,44.0],[-121.5,45.0],[-122.5,45.0],[-122.5,44.0]]]}</v>
@@ -658,7 +658,7 @@
         <v>GeoJSON</v>
       </c>
       <c r="E5" t="str">
-        <v>https://example.com/maps/pacific-nw-forest.geojson</v>
+        <v>https://example.com/maps/sample-forest.geojson</v>
       </c>
       <c r="F5" t="str">
         <v>NEW-3</v>
@@ -703,7 +703,7 @@
         <v>45000</v>
       </c>
       <c r="D2" t="str">
-        <v>EST-VCS-2024-001-Y1</v>
+        <v>SAMPLE-EST-PRJ1-Y1</v>
       </c>
       <c r="E2" t="str">
         <v>NEW-1</v>
@@ -720,7 +720,7 @@
         <v>52000</v>
       </c>
       <c r="D3" t="str">
-        <v>EST-VCS-2024-001-Y2</v>
+        <v>SAMPLE-EST-PRJ1-Y2</v>
       </c>
       <c r="E3" t="str">
         <v>NEW-1</v>
@@ -737,7 +737,7 @@
         <v>58000.5</v>
       </c>
       <c r="D4" t="str">
-        <v>EST-VCS-2024-001-Y3</v>
+        <v>SAMPLE-EST-PRJ1-Y3</v>
       </c>
       <c r="E4" t="str">
         <v>NEW-1</v>
@@ -754,7 +754,7 @@
         <v>12500</v>
       </c>
       <c r="D5" t="str">
-        <v>EST-GS-10542-Y1</v>
+        <v>SAMPLE-EST-PRJ2-Y1</v>
       </c>
       <c r="E5" t="str">
         <v>NEW-2</v>
@@ -771,7 +771,7 @@
         <v>95000.25</v>
       </c>
       <c r="D6" t="str">
-        <v>EST-CAR-2025-078-Y1</v>
+        <v>SAMPLE-EST-PRJ3-Y1</v>
       </c>
       <c r="E6" t="str">
         <v>NEW-3</v>
@@ -810,13 +810,13 @@
         <v>CDP</v>
       </c>
       <c r="B2" t="str">
-        <v>CDP Climate Score 2024</v>
+        <v>Sample Climate Score 2024</v>
       </c>
       <c r="C2" t="str">
         <v>A-</v>
       </c>
       <c r="D2" t="str">
-        <v>https://www.cdp.net/scores/2024/vcs-2024-001</v>
+        <v>https://example.com/ratings/sample-prj-2024-001</v>
       </c>
       <c r="E2" t="str">
         <v>NEW-1</v>
@@ -827,13 +827,13 @@
         <v>CCQI</v>
       </c>
       <c r="B3" t="str">
-        <v>CCQI Quality Rating</v>
+        <v>Sample Quality Rating</v>
       </c>
       <c r="C3" t="str">
         <v>4.2</v>
       </c>
       <c r="D3" t="str">
-        <v>https://carboncreditquality.org/ratings/vcs-2024-001</v>
+        <v>https://example.com/ratings/sample-prj-2024-001-ccqi</v>
       </c>
       <c r="E3" t="str">
         <v>NEW-1</v>
@@ -844,7 +844,7 @@
         <v>CDP</v>
       </c>
       <c r="B4" t="str">
-        <v>CDP Climate Score 2024</v>
+        <v>Sample Climate Score 2024</v>
       </c>
       <c r="C4" t="str">
         <v>B</v>
@@ -980,13 +980,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>VAL-VCS-2024-001</v>
+        <v>SAMPLE-VAL-001</v>
       </c>
       <c r="B2" t="str">
         <v>Validation of Project Design Document</v>
       </c>
       <c r="C2" t="str">
-        <v>SCS Global Services</v>
+        <v>Example Validation Services A</v>
       </c>
       <c r="D2" t="str">
         <v>2023-11-15</v>
@@ -1003,13 +1003,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>VAL-GS-10542</v>
+        <v>SAMPLE-VAL-002</v>
       </c>
       <c r="B3" t="str">
         <v>Validation of Project Design Document</v>
       </c>
       <c r="C3" t="str">
-        <v>AENOR International S.A.U.</v>
+        <v>Example Validation Services B</v>
       </c>
       <c r="D3" t="str">
         <v>2024-06-01</v>
@@ -1026,13 +1026,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>VAL-CAR-2025-078</v>
+        <v>SAMPLE-VAL-003</v>
       </c>
       <c r="B4" t="str">
         <v>Validation of Renewal of Credit Period</v>
       </c>
       <c r="C4" t="str">
-        <v>ERM Certification and Verification Services Limited</v>
+        <v>Example Validation Services C</v>
       </c>
       <c r="D4" t="str">
         <v>2024-12-01</v>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>VER-VCS-2024-001-01</v>
+        <v>SAMPLE-VER-001</v>
       </c>
       <c r="B2" t="str">
         <v>2024-01-01</v>
@@ -1089,7 +1089,7 @@
         <v>2024-12-31</v>
       </c>
       <c r="D2" t="str">
-        <v>SCS Global Services</v>
+        <v>Example Validation Services A</v>
       </c>
       <c r="E2" t="str">
         <v>NEW-1</v>
@@ -1100,7 +1100,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>VER-GS-10542-01</v>
+        <v>SAMPLE-VER-002</v>
       </c>
       <c r="B3" t="str">
         <v>2024-06-01</v>
@@ -1109,7 +1109,7 @@
         <v>2025-05-31</v>
       </c>
       <c r="D3" t="str">
-        <v>AENOR International S.A.U.</v>
+        <v>Example Validation Services B</v>
       </c>
       <c r="E3" t="str">
         <v>NEW-2</v>
@@ -1117,7 +1117,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>VER-CAR-2025-078-01</v>
+        <v>SAMPLE-VER-003</v>
       </c>
       <c r="B4" t="str">
         <v>2025-01-01</v>
@@ -1126,7 +1126,7 @@
         <v>2025-12-31</v>
       </c>
       <c r="D4" t="str">
-        <v>ERM Certification and Verification Services Limited</v>
+        <v>Example Validation Services C</v>
       </c>
       <c r="E4" t="str">
         <v>NEW-3</v>
@@ -1168,7 +1168,7 @@
         <v>2024-01-15</v>
       </c>
       <c r="D2" t="str">
-        <v>AR-ACM0003: Afforestation and reforestation of degraded mangrove habitats — applied to coastal zones with verified baseline deforestation rates.</v>
+        <v>Example methodology: Afforestation and reforestation of degraded mangrove habitats — sample description for CADT import testing.</v>
       </c>
     </row>
     <row r="3">
@@ -1182,7 +1182,7 @@
         <v>2025-01-10</v>
       </c>
       <c r="D3" t="str">
-        <v>VM0012: Improved Forest Management in Temperate and Boreal Forests — extended rotation and selective harvest approach.</v>
+        <v>Example methodology: Improved Forest Management in Temperate and Boreal Forests — sample description for CADT import testing.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: add missing PK columns to sample XLSX fixtures
The projects and units sheets were missing their primary key columns
(cadTrustProjectId / cadTrustUnitId). This caused transformMetaUid to
assign UUIDs to child FK references that didn't match the parent rows,
breaking parent-child linkage on import.

Add fixture-validation integration tests that parse the sample XLSX
files and verify FK consistency, so this class of bug is caught by
the fast test suite going forward.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/tests/v2/live-api/data/sample-projects-import.xlsx
+++ b/tests/v2/live-api/data/sample-projects-import.xlsx
@@ -405,160 +405,172 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>cadTrustProjectId</v>
+      </c>
+      <c r="B1" t="str">
         <v>projectRegistryName</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>projectId</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>projectCreditingProgram</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>projectName</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>projectLink</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>projectDescription</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>projectSector</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>projectType</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>projectSubtype</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>projectStatus</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>projectStatusDate</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>projectUnitMetric</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>cadTrustProgramId</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>NEW-1</v>
+      </c>
+      <c r="B2" t="str">
         <v>Sample Global Registry</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>SAMPLE-PRJ-2024-001</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Example Crediting Program A</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Example Mangrove Restoration Project</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>https://example.com/registry/projects/sample-prj-2024-001</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Sample large-scale mangrove restoration project for testing purposes. This fictional project demonstrates a reforestation scenario with community-based sustainable aquaculture across an example coastal region.</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>["Afforestation and reforestation"]</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>["Afforestation","Reforestation"]</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Mangrove Restoration</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Registered</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>2024-03-15</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>tCO2e</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>NEW-2</v>
+      </c>
+      <c r="B3" t="str">
         <v>Example Standards Body</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>SAMPLE-PRJ-2024-002</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Sample Solar Cookstove Distribution</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>https://example.com/registry/projects/sample-prj-2024-002</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>["Energy demand"]</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>["Solar"]</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Validated</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>2024-08-01</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>tCO2e</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>NEW-3</v>
+      </c>
+      <c r="B4" t="str">
         <v>Example Forestry Registry</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>SAMPLE-PRJ-2025-003</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Example Crediting Program B</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Example Improved Forest Management</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>https://example.com/registry/projects/sample-prj-2025-003</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Sample improved forest management project for testing. This fictional project demonstrates extended rotations and selective thinning in a mixed-conifer forest scenario for CADT import/export testing.</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>["Afforestation and reforestation","Agriculture"]</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>["Agriculture, forestry and other land use (AFOLU)"]</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Improved Forest Management</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>Listed</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>2025-01-10</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>tCO2e</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>{{PROGRAM_ID}}</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>